<commit_message>
Crawlability audit: third verification round wording fixes
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/crawlability-anbar-september-2026.xlsx
+++ b/public/crawlability-anbar-september-2026.xlsx
@@ -1308,7 +1308,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>קישור פנימי לכתובת שמפנה (301). לעדכן את הקישורים הפנימיים ישירות לכתובת היעד.</t>
+          <t>הכתובת מפנה לעמוד הבית: העמוד המקורי הוסר. לשחזר את העמוד או לעדכן את הקישור לעמוד רלוונטי; אין להשאיר קישורים שמובילים לעמוד הבית דרך הפניה.</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>קישור פנימי לכתובת שמפנה (301). לעדכן את הקישורים הפנימיים ישירות לכתובת היעד.</t>
+          <t>הכתובת מפנה לעמוד הבית: העמוד המקורי הוסר. לשחזר את העמוד או לעדכן את הקישור לעמוד רלוונטי; אין להשאיר קישורים שמובילים לעמוד הבית דרך הפניה.</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">

</xml_diff>